<commit_message>
fix(auth): always show Google account chooser on sign-in
Adds prompt:"select_account" to GoogleAuthProvider so the account picker
appears even when a Google session is already active, letting the teacher
choose which account's data to load. Also removes HEDY NG YEE TONG from
the PBD BI dataset and updates the namelist reference spreadsheet.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pupils-tracker/docs/References/namelist.xlsx
+++ b/pupils-tracker/docs/References/namelist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Claude\Pupils-tracker\pupils-tracker\docs\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700D3C42-8528-46DC-BD23-DD01C3559D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4D08A7-DF3F-471D-B17E-962F4594E9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>CHIN YU KAI</t>
   </si>
@@ -572,6 +572,15 @@
   </si>
   <si>
     <t>YUNA BANG PEI RAN</t>
+  </si>
+  <si>
+    <t>DORCAS LU XIN XUAN</t>
+  </si>
+  <si>
+    <t>JORDAN GOO JUN YANG</t>
+  </si>
+  <si>
+    <t>FELIX CHAI JIN ZHE</t>
   </si>
 </sst>
 </file>
@@ -667,16 +676,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -966,337 +975,367 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>37</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="4"/>
+      <c r="C37" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
@@ -1304,36 +1343,6 @@
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1348,333 +1357,352 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -1682,30 +1710,11 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1720,333 +1729,352 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -2054,17 +2082,371 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C4432-C9A3-4195-8DBA-2D4CD25140B2}">
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>38</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C38" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -2072,348 +2454,22 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C4432-C9A3-4195-8DBA-2D4CD25140B2}">
-  <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="4"/>
-    </row>
-    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C14" s="4"/>
-    </row>
-    <row r="15" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C15" s="4"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="4"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C18" s="4"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C21" s="4"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="4"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C23" s="4"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="4"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>25</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C25" s="4"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C26" s="4"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" s="4"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>28</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C28" s="4"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C29" s="4"/>
-    </row>
-    <row r="30" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C30" s="4"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>31</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="4"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>32</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C32" s="4"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>33</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C33" s="4"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>34</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C34" s="4"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C35" s="4"/>
-    </row>
-    <row r="36" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>36</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C36" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="36">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
@@ -2421,35 +2477,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2457,7 +2484,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6E9A3F-E98F-468F-86A1-A43609D2D5AF}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2716,7 +2743,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
@@ -2724,7 +2751,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
@@ -2732,7 +2759,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
@@ -2740,7 +2767,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
@@ -2748,7 +2775,22 @@
         <v>180</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B38" s="1"/>
+      <c r="C38" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B38:C38"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "fix(auth): always show Google account chooser on sign-in"
This reverts commit 4235433f6b999469fbd54131376172a320ad95d1.
</commit_message>
<xml_diff>
--- a/pupils-tracker/docs/References/namelist.xlsx
+++ b/pupils-tracker/docs/References/namelist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Claude\Pupils-tracker\pupils-tracker\docs\References\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4D08A7-DF3F-471D-B17E-962F4594E9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700D3C42-8528-46DC-BD23-DD01C3559D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
   <si>
     <t>CHIN YU KAI</t>
   </si>
@@ -572,15 +572,6 @@
   </si>
   <si>
     <t>YUNA BANG PEI RAN</t>
-  </si>
-  <si>
-    <t>DORCAS LU XIN XUAN</t>
-  </si>
-  <si>
-    <t>JORDAN GOO JUN YANG</t>
-  </si>
-  <si>
-    <t>FELIX CHAI JIN ZHE</t>
   </si>
 </sst>
 </file>
@@ -676,16 +667,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -975,343 +966,361 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="2"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="2"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="2"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="2"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="2"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="4"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>37</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="2"/>
+      <c r="C37" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -1319,30 +1328,12 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1357,328 +1348,357 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="2"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="2"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="2"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C34" s="2"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="2"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1686,35 +1706,6 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1729,328 +1720,357 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="2"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="2"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C33" s="2"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="2"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="2"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="2"/>
+      <c r="C36" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2058,35 +2078,6 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2094,359 +2085,358 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C4432-C9A3-4195-8DBA-2D4CD25140B2}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="2"/>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C4" s="2"/>
+      <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="4"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="2"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C10" s="2"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C11" s="2"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C14" s="2"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="2"/>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C17" s="2"/>
+      <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C19" s="2"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C20" s="2"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C21" s="2"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="C22" s="2"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C24" s="2"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="2"/>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C26" s="2"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C27" s="2"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C28" s="2"/>
+      <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C29" s="2"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C30" s="2"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C31" s="2"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C32" s="2"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="C33" s="2"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C34" s="2"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C35" s="2"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C36" s="2"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>37</v>
-      </c>
-      <c r="B37" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>38</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="C38" s="2"/>
+      <c r="C36" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
+  <mergeCells count="36">
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -2454,29 +2444,12 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2484,7 +2457,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6E9A3F-E98F-468F-86A1-A43609D2D5AF}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2743,7 +2716,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
@@ -2751,7 +2724,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
@@ -2759,7 +2732,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
@@ -2767,7 +2740,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
@@ -2775,22 +2748,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37">
-        <v>37</v>
-      </c>
-      <c r="B37" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B38" s="1"/>
-      <c r="C38" s="2"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B38:C38"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(spelling): persist timer state across fullscreen transitions
Lift ClassTimer state into a shared TimerContext (lib/useTimer.tsx) so the
running countdown survives entering and exiting fullscreen. Previously, entering
Present mode mounted a fresh ClassTimer instance inside the fullscreen element
while the running instance in the Shell toolbar became inaccessible, making the
timer appear to vanish.

Also: re-apply Google account-chooser prompt on sign-in (prompt: select_account),
update namelist.xlsx, and remove a pupil entry from pbd-bi.ts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pupils-tracker/docs/References/namelist.xlsx
+++ b/pupils-tracker/docs/References/namelist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Claude\Pupils-tracker\pupils-tracker\docs\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700D3C42-8528-46DC-BD23-DD01C3559D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4D08A7-DF3F-471D-B17E-962F4594E9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>CHIN YU KAI</t>
   </si>
@@ -572,6 +572,15 @@
   </si>
   <si>
     <t>YUNA BANG PEI RAN</t>
+  </si>
+  <si>
+    <t>DORCAS LU XIN XUAN</t>
+  </si>
+  <si>
+    <t>JORDAN GOO JUN YANG</t>
+  </si>
+  <si>
+    <t>FELIX CHAI JIN ZHE</t>
   </si>
 </sst>
 </file>
@@ -667,16 +676,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -966,337 +975,367 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>37</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="4"/>
+      <c r="C37" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
@@ -1304,36 +1343,6 @@
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1348,333 +1357,352 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -1682,30 +1710,11 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1720,333 +1729,352 @@
       <c r="A1">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="4"/>
+      <c r="C7" s="2"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="2"/>
     </row>
     <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="4"/>
+      <c r="C9" s="2"/>
     </row>
     <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="4"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="4"/>
+      <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="4"/>
+      <c r="C12" s="2"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="2"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="4"/>
+      <c r="C14" s="2"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="4"/>
+      <c r="C15" s="2"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="4"/>
+      <c r="C16" s="2"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="4"/>
+      <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="2"/>
     </row>
     <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>21</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="2"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="2"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>23</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>24</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>25</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>26</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="4"/>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>27</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C27" s="4"/>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>28</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="4"/>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>29</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C29" s="4"/>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>30</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C30" s="4"/>
+      <c r="C30" s="2"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>31</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="4"/>
+      <c r="C31" s="2"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>32</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="4"/>
+      <c r="C32" s="2"/>
     </row>
     <row r="33" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="2"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C34" s="4"/>
+      <c r="C34" s="2"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="4"/>
+      <c r="C35" s="2"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B36" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="4"/>
+      <c r="C36" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
@@ -2054,17 +2082,371 @@
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C4432-C9A3-4195-8DBA-2D4CD25140B2}">
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>38</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C38" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="37">
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -2072,348 +2454,22 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C4432-C9A3-4195-8DBA-2D4CD25140B2}">
-  <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="4"/>
-    </row>
-    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>9</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="4"/>
-    </row>
-    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="4"/>
-    </row>
-    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="4"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="C14" s="4"/>
-    </row>
-    <row r="15" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C15" s="4"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="4"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="C18" s="4"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C19" s="4"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C20" s="4"/>
-    </row>
-    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C21" s="4"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="4"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C23" s="4"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" s="4"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>25</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="C25" s="4"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>26</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C26" s="4"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>27</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" s="4"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>28</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C28" s="4"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C29" s="4"/>
-    </row>
-    <row r="30" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C30" s="4"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>31</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="4"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>32</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C32" s="4"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>33</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="C33" s="4"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>34</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C34" s="4"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>35</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C35" s="4"/>
-    </row>
-    <row r="36" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>36</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C36" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="36">
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
@@ -2421,35 +2477,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2457,7 +2484,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6E9A3F-E98F-468F-86A1-A43609D2D5AF}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2716,7 +2743,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>33</v>
       </c>
@@ -2724,7 +2751,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>34</v>
       </c>
@@ -2732,7 +2759,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>35</v>
       </c>
@@ -2740,7 +2767,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>36</v>
       </c>
@@ -2748,7 +2775,22 @@
         <v>180</v>
       </c>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B38" s="1"/>
+      <c r="C38" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B38:C38"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(roster): add LAI GUN YAU to class 2F
Sync the updated namelist into the app, bump 2F class size to 37, and auto-pull missing roster pupils after hydrate.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pupils-tracker/docs/References/namelist.xlsx
+++ b/pupils-tracker/docs/References/namelist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Claude\Pupils-tracker\pupils-tracker\docs\References\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4D08A7-DF3F-471D-B17E-962F4594E9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DD9EA5-7945-4F24-8A7E-2C853E4C8797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2B" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="185">
   <si>
     <t>CHIN YU KAI</t>
   </si>
@@ -581,6 +581,9 @@
   </si>
   <si>
     <t>FELIX CHAI JIN ZHE</t>
+  </si>
+  <si>
+    <t>LAI GUN YAU</t>
   </si>
 </sst>
 </file>
@@ -1306,12 +1309,25 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
@@ -1324,25 +1340,12 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1679,6 +1682,30 @@
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -1691,6 +1718,362 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D289027-C85A-45A7-89B7-54EDE8949BE3}">
+  <dimension ref="A1:C37"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>30</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>31</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>36</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>37</v>
+      </c>
+      <c r="B37" t="s">
+        <v>184</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="36">
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -1703,354 +2086,6 @@
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D289027-C85A-45A7-89B7-54EDE8949BE3}">
-  <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>5</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>6</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>7</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>8</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>9</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>11</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>12</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>13</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>14</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>15</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>16</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>17</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>22</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>23</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="2"/>
-    </row>
-    <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>24</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>25</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="2"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>26</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C26" s="2"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>27</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>28</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C28" s="2"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>29</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="2"/>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>30</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C30" s="2"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>31</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>32</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>33</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>34</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C34" s="2"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>35</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C35" s="2"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>36</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C36" s="2"/>
-    </row>
-  </sheetData>
-  <mergeCells count="36">
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
@@ -2063,30 +2098,6 @@
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2440,6 +2451,27 @@
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B1:C1"/>
@@ -2456,27 +2488,6 @@
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>